<commit_message>
huga test data refactor
</commit_message>
<xml_diff>
--- a/tests/resources/data.xlsx
+++ b/tests/resources/data.xlsx
@@ -5,13 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="List 1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="Sheet4" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
   <si>
     <t xml:space="preserve">Product ID</t>
   </si>
@@ -73,25 +72,91 @@
     <t xml:space="preserve">OnlineP</t>
   </si>
   <si>
-    <t xml:space="preserve">P-300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-303</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keyboard, Mechanical, RGB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB Cable, 3ft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Online</t>
+    <t xml:space="preserve">Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dulce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abril</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Female</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United States</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hashimoto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great Britain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Philip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kathleen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hanner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nereida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaston</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brumm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hurn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Earlean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melgar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vincenza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weiland</t>
   </si>
 </sst>
 </file>
@@ -201,7 +266,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="12.7421875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.77734375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -289,77 +354,207 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="B6" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="B7" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="n">
-        <v>89.99</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="B9" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>150</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>5.99</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>15</v>
+      <c r="B10" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -379,7 +574,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B3:F7"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
@@ -449,95 +644,6 @@
       </c>
       <c r="F7" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>89.99</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>150</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>5.99</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(): api changes and complete tests refactor (#15)
* complete tests refactor
* api changes and docs
</commit_message>
<xml_diff>
--- a/tests/resources/data.xlsx
+++ b/tests/resources/data.xlsx
@@ -8,21 +8,21 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="List 1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
   <si>
     <t xml:space="preserve">Product ID</t>
   </si>
@@ -42,9 +42,6 @@
     <t xml:space="preserve">Wireless Mouse</t>
   </si>
   <si>
-    <t xml:space="preserve">25.50</t>
-  </si>
-  <si>
     <t xml:space="preserve">Warehouse A, Shelf 2</t>
   </si>
   <si>
@@ -54,9 +51,6 @@
     <t xml:space="preserve">Keyboard, Mechanical</t>
   </si>
   <si>
-    <t xml:space="preserve">89.99</t>
-  </si>
-  <si>
     <t xml:space="preserve">Store Front</t>
   </si>
   <si>
@@ -66,9 +60,6 @@
     <t xml:space="preserve">Monitor 24-inch</t>
   </si>
   <si>
-    <t xml:space="preserve">150.00</t>
-  </si>
-  <si>
     <t xml:space="preserve">Paris, France</t>
   </si>
   <si>
@@ -78,22 +69,94 @@
     <t xml:space="preserve">USB Cable</t>
   </si>
   <si>
-    <t xml:space="preserve">5.99</t>
-  </si>
-  <si>
     <t xml:space="preserve">OnlineP</t>
   </si>
   <si>
-    <t xml:space="preserve">P-300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-303</t>
+    <t xml:space="preserve">Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dulce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abril</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Female</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United States</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hashimoto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great Britain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Philip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kathleen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hanner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nereida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaston</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brumm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hurn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Earlean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melgar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vincenza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weiland</t>
   </si>
 </sst>
 </file>
@@ -203,9 +266,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.77734375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -219,60 +282,60 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="1" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="n">
+        <v>89.99</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="C4" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="C5" s="1" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -291,77 +354,207 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B6" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B7" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="B8" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
+      <c r="B10" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -369,8 +562,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -381,9 +574,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B3:F7"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -397,60 +590,60 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="1" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="n">
+        <v>89.99</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="1" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="1" t="s">
+      <c r="E6" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="1" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="E7" s="1" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -458,8 +651,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>